<commit_message>
正式網域：tbd-web.vercel.app → tbd-edu.com，compass → app.tbd-edu.com
- astro.config.mjs site／sitemap、site.ts siteUrl 與 ogImage、prebuild 的 llms.txt 網址、robots.txt
- pricing.ts COMPASS_URL、vercel.json 兩條 compass 轉址、verify.mjs 的斷言
- 靜態頁 portfolio-guide／grad-path-quiz 的 canonical 與 OG
- 62 份模板 md/csv 與 12 份 xlsx 內文（模板仍經 /pages/placement.html 轉址，D-007 不變）
- library-snapshot.json 的兩個文章連結（正本在 Google Sheet 第 6 欄，需另外改）

舊網域保留 301，已下載的模板連結仍有效。docs/ 與 README 的歷史紀錄不改。

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/assets/templates/grad-agriculture-portfolio-checklist.xlsx
+++ b/public/assets/templates/grad-agriculture-portfolio-checklist.xlsx
@@ -398,13 +398,13 @@
     <t>檢查一下是不是這段時間都在寫內容、沒有回頭處理缺口。內容寫得再多，缺的那幾項還是缺。</t>
   </si>
   <si>
-    <t>搭配文章：農生環境備審怎麼準備？CV、自傳與成果整理　https://tbd-web.vercel.app/pages/resources/agriculture-graduate-cv.html?utm_source=tbd-web&amp;utm_medium=template&amp;utm_campaign=grad-agriculture-portfolio-checklist</t>
+    <t>搭配文章：農生環境備審怎麼準備？CV、自傳與成果整理　https://tbd-edu.com/pages/resources/agriculture-graduate-cv.html?utm_source=tbd-web&amp;utm_medium=template&amp;utm_campaign=grad-agriculture-portfolio-checklist</t>
   </si>
   <si>
     <t>上一階段是研究計畫書、下一階段是口試。備審的主軸由研究計畫決定，備審裡的每一項又都是口試的追問起點。</t>
   </si>
   <si>
-    <t>TBD Studio ｜ 研究所申請陪跑計畫　https://tbd-web.vercel.app/pages/resources/tools.html</t>
+    <t>TBD Studio ｜ 研究所申請陪跑計畫　https://tbd-edu.com/pages/resources/tools.html</t>
   </si>
   <si>
     <t>唯一要寫字的地方，而且只寫關鍵字。這頁是後面打勾的依據，完整文字版在另外幾份表。</t>

</xml_diff>